<commit_message>
Snapshot deployed production v57b before v60 release review
</commit_message>
<xml_diff>
--- a/public/templates/bank-accounts-template.xlsx
+++ b/public/templates/bank-accounts-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="حساب‌ها" sheetId="1" r:id="Rc87b6040b8144d19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="راهنما" sheetId="2" r:id="R917c402f36354950"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="حساب‌ها" sheetId="1" r:id="R2b75a461499c4cd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="راهنما" sheetId="2" r:id="R001743da918a4247"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3356,7 +3356,7 @@
   </x:sheetData>
   <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="A2:A201">
-      <x:formula1>"بانک ملت,بانک ملی ایران,بانک تجارت,بانک پاسارگاد,بانک سامان,بانک صادرات ایران,بانک پارسیان,بانک سپه,بانک شهر,بانک آینده,بانک رفاه کارگران,بانک مسکن,بانک کشاورزی"</x:formula1>
+      <x:formula1>INDIRECT("'راهنما'!$D$2:$D$26")</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="G2:G201">
       <x:formula1>"جاری,کوتاه‌مدت,پشتیبان,تنخواه"</x:formula1>
@@ -3378,6 +3378,7 @@
   <x:cols>
     <x:col min="1" max="1" width="29" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="112" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -3387,6 +3388,9 @@
       <x:c r="B1" s="7" t="str">
         <x:v>روش تکمیل</x:v>
       </x:c>
+      <x:c r="D1" s="7" t="str">
+        <x:v>فهرست بانک‌ها</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="11" t="str">
@@ -3395,6 +3399,9 @@
       <x:c r="B2" s="11" t="str">
         <x:v>الزامی؛ از فهرست کشویی انتخاب کنید.</x:v>
       </x:c>
+      <x:c r="D2" t="str">
+        <x:v>بانک ملت</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="11" t="str">
@@ -3403,6 +3410,9 @@
       <x:c r="B3" s="11" t="str">
         <x:v>الزامی؛ نام کوتاه برای شناسایی حساب در پرتال.</x:v>
       </x:c>
+      <x:c r="D3" t="str">
+        <x:v>بانک ملی ایران</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="11" t="str">
@@ -3411,6 +3421,9 @@
       <x:c r="B4" s="11" t="str">
         <x:v>الزامی؛ نام شرکت یا شخص صاحب حساب، مطابق فرم فعلی.</x:v>
       </x:c>
+      <x:c r="D4" t="str">
+        <x:v>بانک تجارت</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="36" customHeight="1">
       <x:c r="A5" s="11" t="str">
@@ -3419,6 +3432,9 @@
       <x:c r="B5" s="11" t="str">
         <x:v>الزامی؛ ۵تا۲۶رقم. سلول باید Text بماند تا صفرهای ابتدایی حذف نشوند.</x:v>
       </x:c>
+      <x:c r="D5" t="str">
+        <x:v>بانک پاسارگاد</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="36" customHeight="1">
       <x:c r="A6" s="11" t="str">
@@ -3427,6 +3443,9 @@
       <x:c r="B6" s="11" t="str">
         <x:v>اختیاری؛ IR و۲۴رقم. متنی، بدون فرمول.</x:v>
       </x:c>
+      <x:c r="D6" t="str">
+        <x:v>بانک سامان</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="36" customHeight="1">
       <x:c r="A7" s="11" t="str">
@@ -3435,6 +3454,9 @@
       <x:c r="B7" s="11" t="str">
         <x:v>اختیاری؛ ۱۶رقم متنی، بدون فرمول.</x:v>
       </x:c>
+      <x:c r="D7" t="str">
+        <x:v>بانک صادرات ایران</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="36" customHeight="1">
       <x:c r="A8" s="11" t="str">
@@ -3443,6 +3465,9 @@
       <x:c r="B8" s="11" t="str">
         <x:v>اختیاری؛ از فهرست انتخاب کنید. خالی=جاری برای حساب جدید.</x:v>
       </x:c>
+      <x:c r="D8" t="str">
+        <x:v>بانک پارسیان</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="36" customHeight="1">
       <x:c r="A9" s="11" t="str">
@@ -3451,6 +3476,9 @@
       <x:c r="B9" s="11" t="str">
         <x:v>اختیاری.</x:v>
       </x:c>
+      <x:c r="D9" t="str">
+        <x:v>بانک سپه</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="36" customHeight="1">
       <x:c r="A10" s="11" t="str">
@@ -3459,6 +3487,9 @@
       <x:c r="B10" s="11" t="str">
         <x:v>اختیاری؛ رقم متنی با حفظ صفر ابتدایی.</x:v>
       </x:c>
+      <x:c r="D10" t="str">
+        <x:v>بانک شهر</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="57" customHeight="1">
       <x:c r="A11" s="11" t="str">
@@ -3468,6 +3499,9 @@
         <x:v>اختیاری؛ پایا، ساتنا، کارت‌به‌کارت، داخلی، چک. چند روش را با «،» جدا
 کنید. خالی=پایا، ساتنا، کارت‌به‌کارت، داخلی برای حساب جدید.</x:v>
       </x:c>
+      <x:c r="D11" t="str">
+        <x:v>بانک آینده</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="36" customHeight="1">
       <x:c r="A12" s="11" t="str">
@@ -3476,6 +3510,9 @@
       <x:c r="B12" s="11" t="str">
         <x:v>اختیاری؛ فعال/غیرفعال. خالی=فعال برای حساب جدید.</x:v>
       </x:c>
+      <x:c r="D12" t="str">
+        <x:v>بانک رفاه کارگران</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="46" customHeight="1">
       <x:c r="A13" s="11" t="str">
@@ -3485,6 +3522,9 @@
         <x:v>اختیاری؛ بله/خیر. خالی=خیر. پیش‌فرض قبلی تغییر نمی‌کند؛ اگر وجود
 دارد، حساب جدید را «خیر» بزنید.</x:v>
       </x:c>
+      <x:c r="D13" t="str">
+        <x:v>بانک مسکن</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="36" customHeight="1">
       <x:c r="A14" s="11" t="str">
@@ -3493,6 +3533,9 @@
       <x:c r="B14" s="11" t="str">
         <x:v>اختیاری؛ حداکثر۲۰۰۰نویسه.</x:v>
       </x:c>
+      <x:c r="D14" t="str">
+        <x:v>بانک کشاورزی</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="46" customHeight="1">
       <x:c r="A15" s="11" t="str">
@@ -3502,6 +3545,9 @@
         <x:v>شیت «حساب‌ها» را از ردیف۲ پر کنید؛ فقط۲۰۰ردیف. عنوان ستون‌ها را
 تغییر ندهید. شیت راهنما وارد سامانه نمی‌شود.</x:v>
       </x:c>
+      <x:c r="D15" t="str">
+        <x:v>بانک اقتصاد نوین</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="46" customHeight="1">
       <x:c r="A16" s="11" t="str">
@@ -3511,6 +3557,9 @@
         <x:v>ارقام فارسی و انگلیسی پذیرفته‌اند؛ شماره حساب/شبا/کارت/کد شعبه را
 Text وارد کنید. شمارهٔ عددی یا فرمولی پذیرفته نیست.</x:v>
       </x:c>
+      <x:c r="D16" t="str">
+        <x:v>بانک ایران زمین</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="57" customHeight="1">
       <x:c r="A17" s="11" t="str">
@@ -3520,6 +3569,9 @@
         <x:v>تکراری یکسان دوباره ثبت نمی‌شود. اختلاف اطلاعات با حساب موجود یا
 ردیف دیگر خطاست؛ حساب قبلی بازنویسی نمی‌شود.</x:v>
       </x:c>
+      <x:c r="D17" t="str">
+        <x:v>بانک رسالت</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="46" customHeight="1">
       <x:c r="A18" s="11" t="str">
@@ -3529,6 +3581,9 @@
         <x:v>اگر هیچ پیش‌فرضی وجود ندارد، فقط یک حساب جدید فعال می‌تواند صریحاً
 «بله» داشته باشد. حساب‌های قبلی خودکار پیش‌فرض نمی‌شوند.</x:v>
       </x:c>
+      <x:c r="D18" t="str">
+        <x:v>بلوبانک</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="46" customHeight="1">
       <x:c r="A19" s="11" t="str">
@@ -3538,6 +3593,9 @@
         <x:v>فایل را در پرتال انتخاب، نتیجه را بازبینی و سپس ثبت نهایی کنید. تا
 رفع همه خطاها هیچ ردیفی ثبت نمی‌شود.</x:v>
       </x:c>
+      <x:c r="D19" t="str">
+        <x:v>پست بانک ایران</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="36" customHeight="1">
       <x:c r="A20" s="11" t="str">
@@ -3546,10 +3604,41 @@
       <x:c r="B20" s="11" t="str">
         <x:v>فقط xlsx تا۱مگابایت. فایل ماکرو، ناقص یا بیش از۲۰۰ردیف پذیرفته نیست.</x:v>
       </x:c>
+      <x:c r="D20" t="str">
+        <x:v>بانک توسعه تعاون</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="48" customHeight="1">
       <x:c r="A21" s="11"/>
       <x:c r="B21" s="11"/>
+      <x:c r="D21" t="str">
+        <x:v>بانک دی</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="D22" t="str">
+        <x:v>بانک سرمایه</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="D23" t="str">
+        <x:v>بانک سینا</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="D24" t="str">
+        <x:v>بانک قرض‌الحسنه مهر ایران</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="D25" t="str">
+        <x:v>بانک گردشگری</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="D26" t="str">
+        <x:v>مؤسسه اعتباری ملل</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>